<commit_message>
Restore separate knowledge creation entry
</commit_message>
<xml_diff>
--- a/plans/KPBot-Knowledge-任务清单.xlsx
+++ b/plans/KPBot-Knowledge-任务清单.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务清单" sheetId="1" r:id="R70eb92446e2844a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务清单" sheetId="1" r:id="R7fb53a42d88945d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -463,7 +463,7 @@
         <x:v>内置工具代码；KPBot 安装包；依赖锁定；干净安装记录</x:v>
       </x:c>
       <x:c r="F7" s="7" t="str">
-        <x:v>只装 KPBot；更新 Skill 生成三类 Wiki，查询 Skill 独立检索</x:v>
+        <x:v>只装 KPBot；创建 Skill 生成首版，更新 Skill 刷新，查询 Skill 检索</x:v>
       </x:c>
       <x:c r="G7" s="7" t="str">
         <x:v>待开始</x:v>
@@ -989,7 +989,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R259b9bb1f2284e30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b3db618b255405a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>